<commit_message>
Added Auto Update for AMFI
</commit_message>
<xml_diff>
--- a/backend/data/security_master.xlsx
+++ b/backend/data/security_master.xlsx
@@ -11,7 +11,7 @@
     <sheet name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Security Master'!$A$1:$Q$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Security Master'!$A$1:$Q$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q79"/>
+  <dimension ref="A1:Q84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -564,11 +564,7 @@
           <t>Gold Bonds</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>HDFC Focused Fund - Growth Option - Direct Plan</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="b">
@@ -619,11 +615,7 @@
           <t>InvITs</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>HDFC Focused Fund - Growth Option - Direct Plan</t>
-        </is>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="b">
@@ -729,11 +721,7 @@
           <t>REITs</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>HDFC Focused Fund - Growth Option - Direct Plan</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="b">
@@ -1016,23 +1004,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INE00R701025</t>
+          <t>INE238A01034</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>AXIS Bank</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DALBHARAT</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>DALBHARAT.NS</t>
+          <t>AXISBANK.NS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1057,7 +1045,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Dalmia Bharat</t>
+          <t>AXIS Bank</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -1083,23 +1071,23 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INE010V01017</t>
+          <t>INE674K01013</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Aditya Birla Capital</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LTTS</t>
+          <t>ABCAPITAL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>LTTS.NS</t>
+          <t>ABCAPITAL.NS</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1124,7 +1112,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>L&amp;T Technology Services</t>
+          <t>Aditya Birla Capital</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -1150,23 +1138,23 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>INE030A01027</t>
+          <t>INE128X01021</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Archean Chemical Industries</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>ACI</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HINDUNILVR.NS</t>
+          <t>ACI.NS</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1191,7 +1179,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Hindustan Unilever</t>
+          <t>Archean Chemical Industries</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -1217,30 +1205,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>INE040A01034</t>
+          <t>IE000QX7EHP1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>HDFCBANK</t>
-        </is>
-      </c>
+          <t>Ashoka WhiteOak Emerging Markets Equity Ex India Fund Class A</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>HDFCBANK.NS</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>NSE</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>STOCK</t>
@@ -1248,19 +1224,15 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>LRS</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>HDFC Focused Fund - Growth Option - Direct Plan</t>
-        </is>
-      </c>
+          <t>Equity LRS</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="b">
@@ -1272,35 +1244,31 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>RESOLVED</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>YAHOO_FINANCE</t>
-        </is>
-      </c>
+          <t>UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INE048G01026</t>
+          <t>INE406A01037</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Aurobindo Pharma</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>NAVINFLUOR</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>NAVINFLUOR.NS</t>
+          <t>AUROPHARMA.NS</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1325,7 +1293,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Navin Fluorine International</t>
+          <t>Aurobindo Pharma</t>
         </is>
       </c>
       <c r="K15" t="inlineStr"/>
@@ -1351,23 +1319,23 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>INE054A01027</t>
+          <t>INE917I01010</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Bajaj Auto</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>VIPIND</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>VIPIND.NS</t>
+          <t>BAJAJ-AUTO.NS</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1392,7 +1360,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>VIP Industries</t>
+          <t>Bajaj Auto</t>
         </is>
       </c>
       <c r="K16" t="inlineStr"/>
@@ -1418,23 +1386,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>INE062A01020</t>
+          <t>INE296A01032</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Bajaj Finance</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SBIN.NS</t>
+          <t>BAJFINANCE.NS</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1454,12 +1422,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>State Bank Of India</t>
+          <t>Bajaj Finance</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -1485,23 +1453,23 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>INE101D01020</t>
+          <t>INE545U01014</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Bandhan Bank</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>BANDHANBNK</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>GRANULES.NS</t>
+          <t>BANDHANBNK.NS</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1526,7 +1494,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Granules India</t>
+          <t>Bandhan Bank</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
@@ -1552,23 +1520,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>INE121J01017</t>
+          <t>INE397D01024</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Bharti Airtel</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>INDUSTOWER</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>INDUSTOWER.NS</t>
+          <t>BHARTIARTL.NS</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1588,12 +1556,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>HDFC Focused Fund - Growth Option - Direct Plan</t>
+          <t>Bharti Airtel</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
@@ -1619,23 +1587,23 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>INE195A01028</t>
+          <t>INE376G01013</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Biocon Limited</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SUPREMEIND</t>
+          <t>BIOCON</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SUPREMEIND.NS</t>
+          <t>BIOCON.NS</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1660,7 +1628,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Supreme Industries</t>
+          <t>Biocon Limited</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -1686,23 +1654,23 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>INE200M01039</t>
+          <t>INE216A01030</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Britannia Industries</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>VBL</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>VBL.NS</t>
+          <t>BRITANNIA.NS</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1727,7 +1695,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>HDFC Focused Fund - Growth Option - Direct Plan</t>
+          <t>Britannia Industries</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -1753,23 +1721,23 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>INE216A01030</t>
+          <t>INE476A01022</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BRITANNIA.NS</t>
+          <t>CANBK.NS</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1794,7 +1762,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Britannia Industries</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
@@ -1820,23 +1788,23 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>INE238A01034</t>
+          <t>INE136B01020</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Cyient Limited</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>CYIENT</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AXISBANK.NS</t>
+          <t>CYIENT.NS</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1861,7 +1829,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>AXIS Bank</t>
+          <t>Cyient Limited</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -1887,23 +1855,23 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>INE296A01032</t>
+          <t>INE00R701025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Dalmia Bharat</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>DALBHARAT</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BAJFINANCE.NS</t>
+          <t>DALBHARAT.NS</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1928,7 +1896,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Bajaj Finance</t>
+          <t>Dalmia Bharat</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -1954,23 +1922,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>INE399G01023</t>
+          <t>INE148O01028</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>RKFORGE</t>
+          <t>DELHIVERY</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>RKFORGE.NS</t>
+          <t>DELHIVERY.NS</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1995,7 +1963,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Ramkrishna Forgings</t>
+          <t>Delhivery</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -2021,23 +1989,23 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>INE481G01011</t>
+          <t>INE917M01012</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Dilip Buildcon</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>DBL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ULTRACEMCO.NS</t>
+          <t>DBL.NS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2062,7 +2030,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>UltraTech Cement</t>
+          <t>Dilip Buildcon</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -2088,23 +2056,23 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>INE665L01035</t>
+          <t>INE361B01024</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Divi's Laboratories</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>VARROC</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>VARROC.NS</t>
+          <t>DIVISLAB.NS</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2124,12 +2092,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Varroc Engineering</t>
+          <t>Divi's Laboratories</t>
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
@@ -2155,23 +2123,23 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>INE721A01047</t>
+          <t>INE600L01024</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Dr Lal Pathlabs</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>LALPATHLAB</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN.NS</t>
+          <t>LALPATHLAB.NS</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2196,7 +2164,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Shriram Finance</t>
+          <t>Dr Lal Pathlabs</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -2222,23 +2190,23 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>INE765G01017</t>
+          <t>INE089A01031</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Dr. Reddy's Laboratories</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ICICIGI.NS</t>
+          <t>DRREDDY.NS</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2263,7 +2231,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>ICICI Lombard General Insurance Company</t>
+          <t>Dr. Reddy's Laboratories</t>
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
@@ -2289,23 +2257,23 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>INE849A01020</t>
+          <t>INE913H01037</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Endurance Technologies</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>ENDURANCE</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TRENT.NS</t>
+          <t>ENDURANCE.NS</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2330,7 +2298,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Trent Limited</t>
+          <t>Endurance Technologies</t>
         </is>
       </c>
       <c r="K30" t="inlineStr"/>
@@ -2356,23 +2324,23 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>INE917I01010</t>
+          <t>INE068V01023</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Gland Pharma</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>GLAND</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO.NS</t>
+          <t>GLAND.NS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2397,7 +2365,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Bajaj Auto</t>
+          <t>Gland Pharma</t>
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
@@ -2423,23 +2391,23 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>INE917M01012</t>
+          <t>INE159A01016</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>GlaxoSmithkline Pharmaceuticals</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DBL</t>
+          <t>GLAXO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>DBL.NS</t>
+          <t>GLAXO.NS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2464,7 +2432,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Dilip Buildcon</t>
+          <t>GlaxoSmithkline Pharmaceuticals</t>
         </is>
       </c>
       <c r="K32" t="inlineStr"/>
@@ -2490,23 +2458,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>INE918Z01012</t>
+          <t>INE935A01035</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Glenmark Pharmaceuticals</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>KAYNES</t>
+          <t>GLENMARK</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>KAYNES.NS</t>
+          <t>GLENMARK.NS</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2531,7 +2499,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Kaynes Technology India</t>
+          <t>Glenmark Pharmaceuticals</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -2557,23 +2525,23 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>INE935A01035</t>
+          <t>INE101D01020</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Buoyant Opportunities PMS</t>
+          <t>Granules India</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GLENMARK</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>GLENMARK.NS</t>
+          <t>GRANULES.NS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2598,7 +2566,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Glenmark Pharmaceuticals</t>
+          <t>Granules India</t>
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
@@ -2624,23 +2592,23 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>INE018A01030</t>
+          <t>INE860A01027</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>HCL Technologies</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>LT.NS</t>
+          <t>HCLTECH.NS</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2660,12 +2628,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro</t>
+          <t>HCL Technologies</t>
         </is>
       </c>
       <c r="K35" t="inlineStr"/>
@@ -2691,23 +2659,23 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>INE044A01036</t>
+          <t>INE795G01014</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>HDFC Life Insurance Company</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SUNPHARMA.NS</t>
+          <t>HDFCLIFE.NS</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2727,12 +2695,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical</t>
+          <t>HDFC Life Insurance Company</t>
         </is>
       </c>
       <c r="K36" t="inlineStr"/>
@@ -2758,23 +2726,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>INE068V01023</t>
+          <t>INE030A01027</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Hindustan Unilever</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GLAND</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>GLAND.NS</t>
+          <t>HINDUNILVR.NS</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2799,7 +2767,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Gland Pharma</t>
+          <t>Hindustan Unilever</t>
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
@@ -2825,23 +2793,23 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>INE090A01021</t>
+          <t>INE0V6F01027</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Hyundai Motor India</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>HYUNDAI</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ICICIBANK.NS</t>
+          <t>HYUNDAI.NS</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2866,7 +2834,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>ICICI Bank</t>
+          <t>Hyundai Motor India</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -2892,23 +2860,23 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>INE136B01020</t>
+          <t>INE090A01021</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>ICICI Bank</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CYIENT</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>CYIENT.NS</t>
+          <t>ICICIBANK.NS</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2933,7 +2901,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Cyient Limited</t>
+          <t>ICICI Bank</t>
         </is>
       </c>
       <c r="K39" t="inlineStr"/>
@@ -2959,23 +2927,23 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>INE142M01025</t>
+          <t>INE765G01017</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>ICICI Lombard General Insurance Company</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>TATATECH</t>
+          <t>ICICIGI</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>TATATECH.NS</t>
+          <t>ICICIGI.NS</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3000,7 +2968,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Tata Technologies</t>
+          <t>ICICI Lombard General Insurance Company</t>
         </is>
       </c>
       <c r="K40" t="inlineStr"/>
@@ -3026,23 +2994,23 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>INE148O01028</t>
+          <t>INE379A01028</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>ITC Hotels</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>DELHIVERY</t>
+          <t>ITCHOTELS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>DELHIVERY.NS</t>
+          <t>ITCHOTELS.NS</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3062,12 +3030,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Delhivery</t>
+          <t>ITC Hotels</t>
         </is>
       </c>
       <c r="K41" t="inlineStr"/>
@@ -3093,23 +3061,23 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>INE155A01022</t>
+          <t>INE154A01025</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>ITC Limited</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>TMPV.NS</t>
+          <t>ITC.NS</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3129,12 +3097,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Tata Motors Passenger Vehicles</t>
+          <t>ITC Limited</t>
         </is>
       </c>
       <c r="K42" t="inlineStr"/>
@@ -3160,23 +3128,23 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>INE159A01016</t>
+          <t>INE121J01017</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Indus Towers</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>GLAXO</t>
+          <t>INDUSTOWER</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>GLAXO.NS</t>
+          <t>INDUSTOWER.NS</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3201,7 +3169,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>GlaxoSmithkline Pharmaceuticals</t>
+          <t>Indus Towers</t>
         </is>
       </c>
       <c r="K43" t="inlineStr"/>
@@ -3227,23 +3195,23 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>INE160A01022</t>
+          <t>INE009A01021</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>PNB.NS</t>
+          <t>INFY.NS</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3268,7 +3236,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Punjab National Bank</t>
+          <t>Infosys</t>
         </is>
       </c>
       <c r="K44" t="inlineStr"/>
@@ -3294,23 +3262,23 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>INE180A01020</t>
+          <t>INE646L01027</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Interglobe Aviation</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>MFSL</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>MFSL.NS</t>
+          <t>INDIGO.NS</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3335,7 +3303,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Max Financial Services</t>
+          <t>Interglobe Aviation</t>
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
@@ -3361,23 +3329,23 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>INE1TAE01010</t>
+          <t>INE121E01018</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>JSW Energy</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>TMCV</t>
+          <t>JSWENERGY</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>TMCV.NS</t>
+          <t>JSWENERGY.NS</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3397,12 +3365,12 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Tata Motors</t>
+          <t>JSW Energy</t>
         </is>
       </c>
       <c r="K46" t="inlineStr"/>
@@ -3428,23 +3396,23 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>INE205C01021</t>
+          <t>INE880J01026</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>JSW Infrastructure</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>POLYMED</t>
+          <t>JSWINFRA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>POLYMED.NS</t>
+          <t>JSWINFRA.NS</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3464,12 +3432,12 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Poly Medicure</t>
+          <t>JSW Infrastructure</t>
         </is>
       </c>
       <c r="K47" t="inlineStr"/>
@@ -3495,23 +3463,23 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>INE214T01019</t>
+          <t>INE220G01021</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Jindal Stainless</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LTM</t>
+          <t>JSL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>LTM.NS</t>
+          <t>JSL.NS</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3531,12 +3499,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>LTM Limited</t>
+          <t>Jindal Stainless</t>
         </is>
       </c>
       <c r="K48" t="inlineStr"/>
@@ -3562,23 +3530,23 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>INE262H01021</t>
+          <t>INE303R01014</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Kalyan Jewellers India</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PERSISTENT</t>
+          <t>KALYANKJIL</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>PERSISTENT.NS</t>
+          <t>KALYANKJIL.NS</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3603,7 +3571,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Persistent Systems</t>
+          <t>Kalyan Jewellers India</t>
         </is>
       </c>
       <c r="K49" t="inlineStr"/>
@@ -3629,23 +3597,23 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>INE303R01014</t>
+          <t>INE918Z01012</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Kaynes Technology India</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>KALYANKJIL</t>
+          <t>KAYNES</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>KALYANKJIL.NS</t>
+          <t>KAYNES.NS</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3670,7 +3638,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Kalyan Jewellers India</t>
+          <t>Kaynes Technology India</t>
         </is>
       </c>
       <c r="K50" t="inlineStr"/>
@@ -3696,23 +3664,23 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>INE318A01026</t>
+          <t>INE237A01036</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Kotak Mahindra Bank</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>PIDILITIND.NS</t>
+          <t>KOTAKBANK.NS</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3732,12 +3700,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Pidilite Industries</t>
+          <t>Kotak Mahindra Bank</t>
         </is>
       </c>
       <c r="K51" t="inlineStr"/>
@@ -3763,23 +3731,23 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>INE324D01010</t>
+          <t>INE010V01017</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>L&amp;T Technology Services</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>LGEINDIA</t>
+          <t>LTTS</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>LGEINDIA.NS</t>
+          <t>LTTS.NS</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3804,7 +3772,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>LG Electronics India</t>
+          <t>L&amp;T Technology Services</t>
         </is>
       </c>
       <c r="K52" t="inlineStr"/>
@@ -3830,23 +3798,23 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>INE376G01013</t>
+          <t>INE324D01010</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>LG Electronics India</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>BIOCON</t>
+          <t>LGEINDIA</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>BIOCON.NS</t>
+          <t>LGEINDIA.NS</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -3871,7 +3839,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Biocon Limited</t>
+          <t>LG Electronics India</t>
         </is>
       </c>
       <c r="K53" t="inlineStr"/>
@@ -3897,23 +3865,23 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>INE397D01024</t>
+          <t>INE214T01019</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>LTM Limited</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LTM</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>BHARTIARTL.NS</t>
+          <t>LTM.NS</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -3938,7 +3906,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Bharti Airtel</t>
+          <t>LTM Limited</t>
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
@@ -3964,23 +3932,23 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>INE406A01037</t>
+          <t>INE018A01030</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Larsen &amp; Toubro</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>AUROPHARMA.NS</t>
+          <t>LT.NS</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4005,7 +3973,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Aurobindo Pharma</t>
+          <t>Larsen &amp; Toubro</t>
         </is>
       </c>
       <c r="K55" t="inlineStr"/>
@@ -4031,23 +3999,23 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>INE476A01022</t>
+          <t>INE585B01010</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Maruti Suzuki</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>CANBK.NS</t>
+          <t>MARUTI.NS</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4072,7 +4040,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Canara Bank</t>
+          <t>Maruti Suzuki</t>
         </is>
       </c>
       <c r="K56" t="inlineStr"/>
@@ -4098,23 +4066,23 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>INE545U01014</t>
+          <t>INE180A01020</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Max Financial Services</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>BANDHANBNK</t>
+          <t>MFSL</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>BANDHANBNK.NS</t>
+          <t>MFSL.NS</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4139,7 +4107,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Bandhan Bank</t>
+          <t>Max Financial Services</t>
         </is>
       </c>
       <c r="K57" t="inlineStr"/>
@@ -4165,23 +4133,23 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>INE575P01011</t>
+          <t>INE048G01026</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Navin Fluorine International</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>STARHEALTH</t>
+          <t>NAVINFLUOR</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>STARHEALTH.NS</t>
+          <t>NAVINFLUOR.NS</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4206,7 +4174,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Star Health &amp; Allied Insurance Company</t>
+          <t>Navin Fluorine International</t>
         </is>
       </c>
       <c r="K58" t="inlineStr"/>
@@ -4232,23 +4200,23 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>INE585B01010</t>
+          <t>INE982J01020</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>One 97 Communications</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>PAYTM</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>MARUTI.NS</t>
+          <t>PAYTM.NS</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4273,7 +4241,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Maruti Suzuki</t>
+          <t>One 97 Communications</t>
         </is>
       </c>
       <c r="K59" t="inlineStr"/>
@@ -4299,23 +4267,23 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>INE600L01024</t>
+          <t>INE761H01022</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Page Industries</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LALPATHLAB</t>
+          <t>PAGEIND</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
-          <t>LALPATHLAB.NS</t>
+          <t>PAGEIND.NS</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -4340,7 +4308,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Dr Lal Pathlabs</t>
+          <t>Page Industries</t>
         </is>
       </c>
       <c r="K60" t="inlineStr"/>
@@ -4366,23 +4334,23 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>INE646L01027</t>
+          <t>INE262H01021</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Persistent Systems</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>PERSISTENT</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>INDIGO.NS</t>
+          <t>PERSISTENT.NS</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -4407,7 +4375,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Interglobe Aviation</t>
+          <t>Persistent Systems</t>
         </is>
       </c>
       <c r="K61" t="inlineStr"/>
@@ -4433,23 +4401,23 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>INE669C01036</t>
+          <t>INE318A01026</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Pidilite Industries</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
-          <t>TECHM.NS</t>
+          <t>PIDILITIND.NS</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -4474,7 +4442,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Tech Mahindra</t>
+          <t>Pidilite Industries</t>
         </is>
       </c>
       <c r="K62" t="inlineStr"/>
@@ -4500,23 +4468,23 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>INE674K01013</t>
+          <t>INE205C01021</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Poly Medicure</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ABCAPITAL</t>
+          <t>POLYMED</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ABCAPITAL.NS</t>
+          <t>POLYMED.NS</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -4541,7 +4509,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Aditya Birla Capital</t>
+          <t>Poly Medicure</t>
         </is>
       </c>
       <c r="K63" t="inlineStr"/>
@@ -4567,23 +4535,23 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>INE761H01022</t>
+          <t>INE160A01022</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Punjab National Bank</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PAGEIND</t>
+          <t>PNB</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
-          <t>PAGEIND.NS</t>
+          <t>PNB.NS</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -4608,7 +4576,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Page Industries</t>
+          <t>Punjab National Bank</t>
         </is>
       </c>
       <c r="K64" t="inlineStr"/>
@@ -4634,23 +4602,23 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>INE854D01024</t>
+          <t>INE399G01023</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Ramkrishna Forgings</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>UNITDSPR</t>
+          <t>RKFORGE</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>UNITDSPR.NS</t>
+          <t>RKFORGE.NS</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -4675,7 +4643,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>United Spirits</t>
+          <t>Ramkrishna Forgings</t>
         </is>
       </c>
       <c r="K65" t="inlineStr"/>
@@ -4701,23 +4669,23 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>INE913H01037</t>
+          <t>INE423Y01016</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>SBFC Finance</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ENDURANCE</t>
+          <t>SBFC</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ENDURANCE.NS</t>
+          <t>SBFC.NS</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -4737,12 +4705,12 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Equity PMS</t>
+          <t>Direct Equity</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Endurance Technologies</t>
+          <t>SBFC Finance</t>
         </is>
       </c>
       <c r="K66" t="inlineStr"/>
@@ -4768,23 +4736,23 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>INE982J01020</t>
+          <t>INE721A01047</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Carnelian Capital Compounder Strategy</t>
+          <t>Shriram Finance</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>PAYTM</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>PAYTM.NS</t>
+          <t>SHRIRAMFIN.NS</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -4809,7 +4777,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>One 97 Communications</t>
+          <t>Shriram Finance</t>
         </is>
       </c>
       <c r="K67" t="inlineStr"/>
@@ -4835,23 +4803,23 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>INE121E01018</t>
+          <t>INE575P01011</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Star Health &amp; Allied Insurance Company</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>JSWENERGY</t>
+          <t>STARHEALTH</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>JSWENERGY.NS</t>
+          <t>STARHEALTH.NS</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -4871,12 +4839,12 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>JSW Energy</t>
+          <t>Star Health &amp; Allied Insurance Company</t>
         </is>
       </c>
       <c r="K68" t="inlineStr"/>
@@ -4902,23 +4870,23 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>INE154A01025</t>
+          <t>INE062A01020</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>State Bank Of India</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>ITC.NS</t>
+          <t>SBIN.NS</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -4938,12 +4906,12 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>ITC Limited</t>
+          <t>State Bank Of India</t>
         </is>
       </c>
       <c r="K69" t="inlineStr"/>
@@ -4969,23 +4937,23 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>INE220G01021</t>
+          <t>INE044A01036</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Sun Pharmaceutical</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>JSL</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>JSL.NS</t>
+          <t>SUNPHARMA.NS</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5005,12 +4973,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Jindal Stainless</t>
+          <t>Sun Pharmaceutical</t>
         </is>
       </c>
       <c r="K70" t="inlineStr"/>
@@ -5036,23 +5004,23 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>INE237A01036</t>
+          <t>INE195A01028</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Supreme Industries</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>SUPREMEIND</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>KOTAKBANK.NS</t>
+          <t>SUPREMEIND.NS</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5072,12 +5040,12 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Kotak Mahindra Bank</t>
+          <t>Supreme Industries</t>
         </is>
       </c>
       <c r="K71" t="inlineStr"/>
@@ -5103,23 +5071,23 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>INE245A01021</t>
+          <t>INE1TAE01010</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Tata Motors</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>TMCV</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>TATAPOWER.NS</t>
+          <t>TMCV.NS</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5139,12 +5107,12 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Tata Motors</t>
         </is>
       </c>
       <c r="K72" t="inlineStr"/>
@@ -5170,23 +5138,23 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>INE280A01028</t>
+          <t>INE155A01022</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Tata Motors Passenger Vehicles</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
-          <t>TITAN.NS</t>
+          <t>TMPV.NS</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5206,12 +5174,12 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Titan Company</t>
+          <t>Tata Motors Passenger Vehicles</t>
         </is>
       </c>
       <c r="K73" t="inlineStr"/>
@@ -5237,23 +5205,23 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>INE361B01024</t>
+          <t>INE245A01021</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Tata Power</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>TATAPOWER</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>DIVISLAB.NS</t>
+          <t>TATAPOWER.NS</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5278,7 +5246,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Divi's Laboratories</t>
+          <t>Tata Power</t>
         </is>
       </c>
       <c r="K74" t="inlineStr"/>
@@ -5304,23 +5272,23 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>INE379A01028</t>
+          <t>INE142M01025</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Tata Technologies</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ITCHOTELS</t>
+          <t>TATATECH</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ITCHOTELS.NS</t>
+          <t>TATATECH.NS</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -5340,12 +5308,12 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>ITC Hotels</t>
+          <t>Tata Technologies</t>
         </is>
       </c>
       <c r="K75" t="inlineStr"/>
@@ -5371,23 +5339,23 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>INE423Y01016</t>
+          <t>INE669C01036</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Tech Mahindra</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SBFC</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
-          <t>SBFC.NS</t>
+          <t>TECHM.NS</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -5407,12 +5375,12 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>SBFC Finance</t>
+          <t>Tech Mahindra</t>
         </is>
       </c>
       <c r="K76" t="inlineStr"/>
@@ -5438,23 +5406,23 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>INE795G01014</t>
+          <t>INE280A01028</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Titan Company</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
-          <t>HDFCLIFE.NS</t>
+          <t>TITAN.NS</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -5479,7 +5447,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>HDFC Life Insurance Company</t>
+          <t>Titan Company</t>
         </is>
       </c>
       <c r="K77" t="inlineStr"/>
@@ -5505,23 +5473,23 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>INE860A01027</t>
+          <t>INE849A01020</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Trent Limited</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
-          <t>HCLTECH.NS</t>
+          <t>TRENT.NS</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -5541,12 +5509,12 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>HCL Technologies</t>
+          <t>Trent Limited</t>
         </is>
       </c>
       <c r="K78" t="inlineStr"/>
@@ -5572,23 +5540,23 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>INE880J01026</t>
+          <t>INE481G01011</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>UltraTech Cement</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>JSWINFRA</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
-          <t>JSWINFRA.NS</t>
+          <t>ULTRACEMCO.NS</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -5608,12 +5576,12 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Direct Equity</t>
+          <t>Equity PMS</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>JSW Infrastructure</t>
+          <t>UltraTech Cement</t>
         </is>
       </c>
       <c r="K79" t="inlineStr"/>
@@ -5636,8 +5604,343 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>INE854D01024</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>United Spirits</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>UNITDSPR.NS</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Equity PMS</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>United Spirits</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="b">
+        <v>0</v>
+      </c>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="b">
+        <v>1</v>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>YAHOO_FINANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>INE054A01027</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>VIP Industries</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>VIPIND</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>VIPIND.NS</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Equity PMS</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>VIP Industries</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="b">
+        <v>0</v>
+      </c>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="b">
+        <v>1</v>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>YAHOO_FINANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>INE665L01035</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Varroc Engineering</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>VARROC</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>VARROC.NS</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Equity PMS</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Varroc Engineering</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="b">
+        <v>0</v>
+      </c>
+      <c r="N82" t="inlineStr"/>
+      <c r="O82" t="b">
+        <v>1</v>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>YAHOO_FINANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>INE200M01039</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Varun Beverages</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>VBL.NS</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Equity PMS</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Varun Beverages</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="b">
+        <v>0</v>
+      </c>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="b">
+        <v>1</v>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>YAHOO_FINANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>INE1CDF01017</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Vedanta Aluminium Metal</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>VAML</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>VAML.NS</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>NSE</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Equity PMS</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Vedanta Aluminium Metal</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="b">
+        <v>0</v>
+      </c>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="b">
+        <v>1</v>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>YAHOO_FINANCE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q79"/>
+  <autoFilter ref="A1:Q84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5682,12 +5985,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Transaction source</t>
+          <t>Security source</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>D:\PWMS\backend\data\transactions.xlsx</t>
+          <t>Database (Asset/Transaction) - transactions.xlsx is only used as a fallback if present and the database has no ISIN-based securities.</t>
         </is>
       </c>
     </row>

</xml_diff>